<commit_message>
Update DLC chapter overview (id, name, rDate, category, dlcCategories, release, codeName, Folder, Characters).xlsx
</commit_message>
<xml_diff>
--- a/Program/Assets/DLC chapter overview (id, name, rDate, category, dlcCategories, release, codeName, Folder, Characters).xlsx
+++ b/Program/Assets/DLC chapter overview (id, name, rDate, category, dlcCategories, release, codeName, Folder, Characters).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\Perk-Randomiser-for-Dead-by-Daylight\Program\Assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65533A69-15A3-4E7C-8A8F-708A40DC2BEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21ECFE6E-A811-4EDB-BF0E-C2BF5C8ECAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43275" yWindow="2415" windowWidth="24945" windowHeight="12345" xr2:uid="{898976F4-4C52-43AD-8236-3E3A81667028}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="36495" windowHeight="15345" xr2:uid="{898976F4-4C52-43AD-8236-3E3A81667028}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="252">
   <si>
     <t>Cannibal</t>
   </si>
@@ -762,6 +762,36 @@
   </si>
   <si>
     <t>Vee Boonyasak; Krasue</t>
+  </si>
+  <si>
+    <t>Stranger Things Chapter 2</t>
+  </si>
+  <si>
+    <t>27.01.2026</t>
+  </si>
+  <si>
+    <t>9.4.0</t>
+  </si>
+  <si>
+    <t>Poutine</t>
+  </si>
+  <si>
+    <t>Kwon Tae-young</t>
+  </si>
+  <si>
+    <t>9.5.0</t>
+  </si>
+  <si>
+    <t>All-Kill: Comeback</t>
+  </si>
+  <si>
+    <t>17.03.2026</t>
+  </si>
+  <si>
+    <t>TBA</t>
+  </si>
+  <si>
+    <t>Dustin Henderson; Eleven; First</t>
   </si>
 </sst>
 </file>
@@ -1142,7 +1172,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C7EA9D9E-7D72-475F-A94B-28D996D3C3C2}">
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
@@ -1196,7 +1226,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="str">
-        <f t="shared" ref="E2:E48" si="0">CHOOSE(D2, "Chapter DLC", "Half-Chapter DLC", "Clothing Pack DLC", "Original Soundtrack DLC", "Character Pack DLC", "Other", "Retracted", "Chapter Pack DLC")</f>
+        <f t="shared" ref="E2:E50" si="0">CHOOSE(D2, "Chapter DLC", "Half-Chapter DLC", "Clothing Pack DLC", "Original Soundtrack DLC", "Character Pack DLC", "Other", "Retracted", "Chapter Pack DLC")</f>
         <v>Chapter DLC</v>
       </c>
       <c r="F2" t="s">
@@ -2627,9 +2657,69 @@
         <v>241</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>61</v>
+      </c>
+      <c r="B49" t="s">
+        <v>242</v>
+      </c>
+      <c r="C49" t="s">
+        <v>243</v>
+      </c>
+      <c r="D49">
+        <v>1</v>
+      </c>
+      <c r="E49" t="str">
+        <f t="shared" si="0"/>
+        <v>Chapter DLC</v>
+      </c>
+      <c r="F49" t="s">
+        <v>244</v>
+      </c>
+      <c r="G49" t="s">
+        <v>245</v>
+      </c>
+      <c r="H49" t="s">
+        <v>245</v>
+      </c>
+      <c r="I49" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>62</v>
+      </c>
+      <c r="B50" t="s">
+        <v>248</v>
+      </c>
+      <c r="C50" t="s">
+        <v>249</v>
+      </c>
+      <c r="D50">
+        <v>1</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="0"/>
+        <v>Chapter DLC</v>
+      </c>
+      <c r="F50" t="s">
+        <v>247</v>
+      </c>
+      <c r="G50" t="s">
+        <v>250</v>
+      </c>
+      <c r="H50" t="s">
+        <v>250</v>
+      </c>
+      <c r="I50" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>